<commit_message>
fix: no formatting for populating data into the template; minor changes in the excel;
</commit_message>
<xml_diff>
--- a/india_compliance/gst_india/data/GSTR1_Excel_Template_V2.0.xlsx
+++ b/india_compliance/gst_india/data/GSTR1_Excel_Template_V2.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\snv\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDD692DE-45C5-42AE-B241-18E965B17737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA4D2032-6455-415D-B41A-E1ABA9BB6343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="12" activeTab="9" xr2:uid="{41E52190-9EEB-4DD3-ABBA-4CAF8812DBCA}"/>
   </bookViews>
@@ -1989,7 +1989,7 @@
       <c r="F5" s="22"/>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Negative value not allowed. Please enter positive value." sqref="L5:M1048576 E5:E1048576" xr:uid="{2A1457C6-7B6D-4920-82DE-94D7DB82A96C}">
       <formula1>0</formula1>
     </dataValidation>
@@ -2011,6 +2011,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I1048576" xr:uid="{A08FA292-14C4-43E2-9ECA-1E6BB0E9AC42}">
       <formula1>INVTYPE</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K5:K1048576" xr:uid="{E7BD63B0-E267-43AB-925E-C4E6A46E022E}">
+      <formula1>RATE</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>